<commit_message>
DOCS(geometry): Renumber archived arm measurement workbooks
Add the update-1 workbook to the measurement archive.

Rename update-4, update-5, and update-6 to update-2, update-3, and update-4 respectively. Preserve the contents of all three renamed workbooks.
</commit_message>
<xml_diff>
--- a/ProjectDevGuide/docs/archive/arm-measurements/Arm_IK_Measurements-update-4.xlsx
+++ b/ProjectDevGuide/docs/archive/arm-measurements/Arm_IK_Measurements-update-4.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="149">
   <si>
     <t xml:space="preserve">Servo rotation axes - ARM_ASSEMBLY, all joints at 0 deg (arm straight up)</t>
   </si>
@@ -176,19 +176,19 @@
     <t xml:space="preserve">Left jaw tip</t>
   </si>
   <si>
-    <t xml:space="preserve">gripper_part_left max Y</t>
+    <t xml:space="preserve">gripper_part_left max Y at file-open pose. Moves 403-409 with jaw opening</t>
   </si>
   <si>
     <t xml:space="preserve">Right jaw tip</t>
   </si>
   <si>
-    <t xml:space="preserve">gripper_part_right max Y</t>
+    <t xml:space="preserve">gripper_part_right max Y at file-open pose. Moves 403-409 with jaw opening</t>
   </si>
   <si>
     <t xml:space="preserve">Jaw midplane</t>
   </si>
   <si>
-    <t xml:space="preserve">Midway between the two jaw inner faces near the tip (Y 396-405). Jaws close along Z.</t>
+    <t xml:space="preserve">Midway between jaw inner faces. Checked at gear -10/0/10/20 deg: 27.6-28.1 every time, so Z does not depend on jaw opening.</t>
   </si>
   <si>
     <t xml:space="preserve">Jaw thickness centre</t>
@@ -197,13 +197,13 @@
     <t xml:space="preserve">Jaws span X -16.64 .. -3.64 at the tip, centre -10.14</t>
   </si>
   <si>
-    <t xml:space="preserve">Object centre (grip point)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAD. X = jaw thickness centre, Z = jaw midplane. Y uses grip offset in IK Lengths!B11 (OPEN QUESTION)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Object (cube) size</t>
+    <t xml:space="preserve">Object centre (grip point) - CAD, file-open jaw pose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD only. Y = file-open jaw tips avg - 3.5; NOT the measured grip position. X/Z are pose-independent. FK uses FK Geometry!D10 (103.5) for the along-tool distance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object (block) size</t>
   </si>
   <si>
     <t xml:space="preserve">Width, between jaws (Z)</t>
@@ -218,9 +218,6 @@
     <t xml:space="preserve">Length, along the tool axis (Y)</t>
   </si>
   <si>
-    <t xml:space="preserve">Orientation assumed - confirm</t>
-  </si>
-  <si>
     <t xml:space="preserve">Link lengths for inverse kinematics (formulas from the Axes sheet)</t>
   </si>
   <si>
@@ -293,7 +290,7 @@
     <t xml:space="preserve">J5 -&gt; grip point (tool length)</t>
   </si>
   <si>
-    <t xml:space="preserve">Use this as the tool length in IK</t>
+    <t xml:space="preserve">CAD-only tool length for comparison. Use FK Geometry!D10 for the measured-derived tool length (103.5).</t>
   </si>
   <si>
     <t xml:space="preserve">J5-&gt;tip - grip offset</t>
@@ -302,7 +299,7 @@
     <t xml:space="preserve">Grip point back from jaw tip (mm)</t>
   </si>
   <si>
-    <t xml:space="preserve">OPEN: 3.5 gives Y 404.62. If cube face is flush with jaw tips, use 7.5 (half the 15 mm length) -&gt; Y 400.62</t>
+    <t xml:space="preserve">Confirmed: block centre 3.5 mm back from the jaw tip</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -320,7 +317,7 @@
     <t xml:space="preserve">J5 -&gt; object centre, along tool</t>
   </si>
   <si>
-    <t xml:space="preserve">Tool length for FK/IK (CAD)</t>
+    <t xml:space="preserve">CAD only. Tip Y moves with jaw opening, so this is a cross-check, not the value to use</t>
   </si>
   <si>
     <t xml:space="preserve">obj.Y - J5.Y</t>
@@ -383,7 +380,7 @@
     <t xml:space="preserve">J5 Wrist pitch → jaw tip</t>
   </si>
   <si>
-    <t xml:space="preserve">J5 Wrist pitch -&gt; object centre</t>
+    <t xml:space="preserve">J5 Wrist pitch -&gt; object centre (DERIVED: 107 - 3.5)</t>
   </si>
   <si>
     <t xml:space="preserve">How it was measured</t>
@@ -410,10 +407,16 @@
     <t xml:space="preserve">- CAD lengths are within about 1 mm of the print. Larger real-world errors come from servo zero offsets (calibration table) and arm sag / gear backlash.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Object centre: X/Z from jaw geometry in CAD (jaw thickness centre, jaw midplane). Y depends on how deep the cube sits in the jaws.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Gripper jaws in CAD are not perfectly mirrored (tips at Y 409.1 / 407.1), so the midplane is ~27.6, not the gear midplane 29.8.</t>
+    <t xml:space="preserve">- Object centre: X/Z from jaw geometry in CAD (jaw thickness centre, jaw midplane). Y depends on how deep the block sits in the jaws.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Jaw tips in CAD move with the gear angle: tips Y 403.2-405.0 at gear 20 deg, 406.0-407.3 at 10 deg, 408.0-408.7 at 0 deg, 409.1-409.4 at -10 deg (closed). The 409.12/407.12 values came from the file-open state. Tool length therefore uses the ruler measurement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Jaw midplane Z stays 27.6-28.1 at every jaw opening -&gt; 27.7 used. The 29.6-29.8 value is the gear-pivot midplane, not the jaw faces.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Shoulder height (CONDITIONAL): CAD 94.22 is J2 axis above base_plate bottom (Y -34.5). The comparison with the 94 ruler value holds only if the ruler started at the surface the plate sits on.</t>
   </si>
   <si>
     <t xml:space="preserve">Geometry for FK, CAD vs measured. Pick the "Use" column in code.</t>
@@ -458,13 +461,16 @@
     <t xml:space="preserve">J5 -&gt; object centre (along tool)</t>
   </si>
   <si>
-    <t xml:space="preserve">OPEN until grip depth confirmed</t>
+    <t xml:space="preserve">Derived: measured J5-&gt;tip 107 minus 3.5 centre setback (not a direct measurement)</t>
   </si>
   <si>
     <t xml:space="preserve">Object offset X (in J5 frame)</t>
   </si>
   <si>
     <t xml:space="preserve">Object offset Z (from roll axis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD jaw midplane 27.7 - roll axis 33.43</t>
   </si>
 </sst>
 </file>
@@ -578,14 +584,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -638,7 +644,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -675,19 +681,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -703,31 +701,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1311,18 +1305,18 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>53</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>55</v>
       </c>
@@ -1333,30 +1327,30 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G19" s="11" t="n">
+      <c r="G19" s="9" t="n">
         <v>-10.14</v>
       </c>
-      <c r="H19" s="11" t="n">
+      <c r="H19" s="9" t="n">
         <f aca="false">AVERAGE(H15:H16)-'IK Lengths'!B11</f>
         <v>404.62</v>
       </c>
-      <c r="I19" s="11" t="n">
-        <v>27.6</v>
+      <c r="I19" s="9" t="n">
+        <v>27.7</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>60</v>
       </c>
@@ -1367,23 +1361,20 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>62</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>63</v>
       </c>
       <c r="H24" s="1" t="n">
         <v>15</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1413,207 +1404,207 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B4" s="13" t="n">
+        <v>69</v>
+      </c>
+      <c r="B4" s="11" t="n">
         <f aca="false">Axes!H6-Axes!H14</f>
         <v>94.22</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="B5" s="11" t="n">
         <f aca="false">ABS(Axes!G6-Axes!G5)</f>
         <v>23.15</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="B6" s="11" t="n">
         <f aca="false">ABS(Axes!I8-Axes!I5)</f>
         <v>15.25</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="13" t="n">
+        <v>78</v>
+      </c>
+      <c r="B7" s="11" t="n">
         <f aca="false">Axes!H7-Axes!H6</f>
         <v>113.12</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B8" s="13" t="n">
+        <v>81</v>
+      </c>
+      <c r="B8" s="11" t="n">
         <f aca="false">Axes!H9-Axes!H7</f>
         <v>126.4</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="13" t="n">
+        <v>84</v>
+      </c>
+      <c r="B9" s="11" t="n">
         <f aca="false">AVERAGE(Axes!H15:H16)-Axes!H9</f>
         <v>108.88</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>86</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="13" t="n">
+        <v>87</v>
+      </c>
+      <c r="B10" s="11" t="n">
         <f aca="false">B9-B11</f>
         <v>105.38</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D10" s="5" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="B11" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>91</v>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="B16" s="1" t="n">
         <f aca="false">Axes!H19-Axes!H9</f>
         <v>105.38</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D16" s="1" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="B17" s="1" t="n">
         <f aca="false">Axes!G19-Axes!G9</f>
         <v>13</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D17" s="1" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="B18" s="1" t="n">
         <f aca="false">Axes!I19-Axes!I8</f>
-        <v>-5.83</v>
+        <v>-5.73</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D18" s="1" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1642,51 +1633,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" s="17" t="n">
+        <v>114</v>
+      </c>
+      <c r="B6" s="14" t="n">
         <f aca="false">'IK Lengths'!B4</f>
         <v>94.22</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="15" t="n">
         <v>94</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="11" t="n">
         <f aca="false">IF(C6="","",C6-B6)</f>
         <v>-0.219999999999999</v>
       </c>
@@ -1697,16 +1688,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="B7" s="17" t="n">
+        <v>115</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <f aca="false">'IK Lengths'!B7</f>
         <v>113.12</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="15" t="n">
         <v>114</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="11" t="n">
         <f aca="false">IF(C7="","",C7-B7)</f>
         <v>0.879999999999996</v>
       </c>
@@ -1717,16 +1708,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="17" t="n">
+        <v>116</v>
+      </c>
+      <c r="B8" s="14" t="n">
         <f aca="false">'IK Lengths'!B8</f>
         <v>126.4</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="15" t="n">
         <v>127</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="11" t="n">
         <f aca="false">IF(C8="","",C8-B8)</f>
         <v>0.599999999999994</v>
       </c>
@@ -1737,16 +1728,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="B9" s="17" t="n">
+        <v>117</v>
+      </c>
+      <c r="B9" s="14" t="n">
         <f aca="false">'IK Lengths'!B9</f>
         <v>108.88</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="15" t="n">
         <v>107</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">IF(C9="","",C9-B9)</f>
         <v>-1.88</v>
       </c>
@@ -1755,22 +1746,25 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B10" s="17" t="n">
+        <v>118</v>
+      </c>
+      <c r="B10" s="14" t="n">
         <f aca="false">'IK Lengths'!B16</f>
         <v>105.38</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="13" t="str">
+      <c r="C10" s="1" t="n">
+        <f aca="false">'FK Geometry'!C10</f>
+        <v>103.5</v>
+      </c>
+      <c r="D10" s="11" t="n">
         <f aca="false">IF(C10="","",C10-B10)</f>
-        <v/>
+        <v>-1.88</v>
       </c>
       <c r="E10" s="5" t="str">
         <f aca="false">IF(C10="","",IF(ABS(D10)&gt;$B$3,"CHECK","OK"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1792,7 +1786,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="140"/>
@@ -1800,55 +1794,65 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>123</v>
-      </c>
-    </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14"/>
+      <c r="A5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1870,202 +1874,209 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" s="21" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="B3" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="D3" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="E3" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="F3" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="B4" s="22" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="18" t="n">
         <f aca="false">'IK Lengths'!B4</f>
         <v>94.22</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="19" t="n">
         <v>94</v>
       </c>
-      <c r="D4" s="22" t="n">
+      <c r="D4" s="18" t="n">
         <f aca="false">IF(E4="measured",C4,B4)</f>
         <v>94</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>136</v>
-      </c>
-      <c r="F4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="22" t="n">
+      <c r="F4" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="18" t="n">
         <f aca="false">'IK Lengths'!B5</f>
         <v>23.15</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="18" t="n">
         <f aca="false">IF(E5="measured",C5,B5)</f>
         <v>23.15</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="F5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="22" t="n">
+      <c r="F5" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <f aca="false">'IK Lengths'!B6</f>
         <v>15.25</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="18" t="n">
         <f aca="false">IF(E6="measured",C6,B6)</f>
         <v>15.25</v>
       </c>
-      <c r="E6" s="0" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="B7" s="22" t="n">
+      <c r="E6" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="18" t="n">
         <f aca="false">'IK Lengths'!B7</f>
         <v>113.12</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="19" t="n">
         <v>114</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="18" t="n">
         <f aca="false">IF(E7="measured",C7,B7)</f>
         <v>114</v>
       </c>
-      <c r="E7" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="B8" s="22" t="n">
+      <c r="E7" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="18" t="n">
         <f aca="false">'IK Lengths'!B8</f>
         <v>126.4</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="19" t="n">
         <v>127</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="18" t="n">
         <f aca="false">IF(E8="measured",C8,B8)</f>
         <v>127</v>
       </c>
-      <c r="E8" s="0" t="s">
-        <v>136</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="22" t="n">
+      <c r="E8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="18" t="n">
         <f aca="false">'IK Lengths'!B9</f>
         <v>108.88</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="19" t="n">
         <v>107</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="18" t="n">
         <f aca="false">IF(E9="measured",C9,B9)</f>
         <v>107</v>
       </c>
-      <c r="E9" s="0" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="B10" s="22" t="n">
+      <c r="E9" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" s="18" t="n">
         <f aca="false">'IK Lengths'!B16</f>
         <v>105.38</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="C10" s="1" t="n">
+        <f aca="false">C9-'IK Lengths'!B11</f>
+        <v>103.5</v>
+      </c>
+      <c r="D10" s="18" t="n">
         <f aca="false">IF(E10="measured",C10,B10)</f>
-        <v>105.38</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+        <v>103.5</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="22" t="n">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B11" s="18" t="n">
         <f aca="false">'IK Lengths'!B17</f>
         <v>13</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D11" s="18" t="n">
         <f aca="false">IF(E11="measured",C11,B11)</f>
         <v>13</v>
       </c>
-      <c r="E11" s="0" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="B12" s="22" t="n">
+      <c r="E11" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" s="18" t="n">
         <f aca="false">'IK Lengths'!B18</f>
-        <v>-5.83</v>
-      </c>
-      <c r="D12" s="22" t="n">
+        <v>-5.73</v>
+      </c>
+      <c r="D12" s="18" t="n">
         <f aca="false">IF(E12="measured",C12,B12)</f>
-        <v>-5.83</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>138</v>
+        <v>-5.73</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>